<commit_message>
excel based test execution
</commit_message>
<xml_diff>
--- a/src/test/resources/testData.xlsx
+++ b/src/test/resources/testData.xlsx
@@ -3,19 +3,20 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr/>
   <bookViews>
-    <workbookView activeTab="2" tabRatio="500"/>
+    <workbookView tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" name="login" sheetId="1"/>
     <sheet r:id="rId2" name="addToCart" sheetId="2"/>
     <sheet r:id="rId3" name="checkout" sheetId="3"/>
+    <sheet r:id="rId4" name="Sheet4" sheetId="4"/>
   </sheets>
   <calcPr calcId="0" iterate="1" iterateCount="1000" iterateDelta="0.01"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="139">
   <si>
     <t>caseId</t>
   </si>
@@ -86,9 +87,6 @@
     <t>Invalid short mobile number is rejected</t>
   </si>
   <si>
-    <t>12345</t>
-  </si>
-  <si>
     <t>L005</t>
   </si>
   <si>
@@ -131,16 +129,13 @@
     <t>Long invalid mobile number is rejected</t>
   </si>
   <si>
-    <t>999999999999999</t>
-  </si>
-  <si>
     <t>L010</t>
   </si>
   <si>
     <t>Existing-user path can advance to password when valid credentials are supplied by tester</t>
   </si>
   <si>
-    <t>REPLACE_WITH_VALID_AMAZON_EMAIL</t>
+    <t>mugunthannagalingam17@gmail.com</t>
   </si>
   <si>
     <t>PASSWORD_STEP</t>
@@ -444,7 +439,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3">
+  <fonts count="6">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -460,14 +455,29 @@
       <name val="Carlito"/>
     </font>
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
       <b/>
       <i val="0"/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Carlito"/>
     </font>
+    <font>
+      <color auto="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Carlito"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -479,8 +489,13 @@
         <fgColor rgb="FF232F3E"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC0E6F5"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -488,23 +503,20 @@
       <bottom/>
     </border>
     <border>
-      <left>
-        <color rgb="FF000000"/>
+      <left style="thin">
+        <color theme="4" tint="0.2"/>
       </left>
-      <right>
-        <color rgb="FF000000"/>
-      </right>
-      <top>
-        <color rgb="FF000000"/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.2"/>
       </top>
-      <bottom>
-        <color rgb="FF000000"/>
+      <bottom style="thin">
+        <color theme="4" tint="0.2"/>
       </bottom>
     </border>
     <border>
-      <left style="thin">
-        <color theme="4" tint="0.2"/>
-      </left>
+      <left/>
+      <right/>
       <top style="thin">
         <color theme="4" tint="0.2"/>
       </top>
@@ -514,31 +526,94 @@
     </border>
     <border>
       <left style="thin">
-        <color theme="4" tint="0.2"/>
+        <color rgb="FF1F8FBE"/>
       </left>
-      <right>
-        <color rgb="FF000000"/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF1F8FBE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF1F8FBE"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF1F8FBE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF1F8FBE"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF1F8FBE"/>
       </right>
       <top style="thin">
-        <color theme="4" tint="0.2"/>
+        <color rgb="FF1F8FBE"/>
       </top>
       <bottom style="thin">
-        <color theme="4" tint="0.2"/>
+        <color rgb="FF1F8FBE"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF1F8FBE"/>
+      </left>
+      <top style="thin">
+        <color rgb="FF1F8FBE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF1F8FBE"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="FF1F8FBE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF1F8FBE"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="FF1F8FBE"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF1F8FBE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF1F8FBE"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0">
+  <cellXfs count="18">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="1"/>
@@ -866,7 +941,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{C8E28F7C-5EBA-4CE2-A3CD-B0BDE9CBC073}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{0C37B574-ACD3-4DE9-8CD6-49383E9FAEAE}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -879,22 +954,22 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -916,186 +991,187 @@
       </c>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E3" t="s">
+      <c r="D3" s="4"/>
+      <c r="E3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="5" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" t="s">
+      <c r="A4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="8" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" t="s">
+      <c r="A5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="3">
+        <v>12345</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E5" t="s">
+      <c r="B6" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F6" s="8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1">
-      <c r="A6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" t="s">
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D6" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="D7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F7" s="5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="A7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" t="s">
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D7" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" t="s">
+      <c r="D8" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F8" s="8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1">
-      <c r="A8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" t="s">
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D8" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" t="s">
+      <c r="D9" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F9" s="5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1">
-      <c r="A9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B9" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" t="s">
+    <row r="10" ht="15" customHeight="1">
+      <c r="A10" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E9" t="s">
+      <c r="D10" s="7">
+        <v>999999999999999</v>
+      </c>
+      <c r="E10" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F10" s="8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
-      <c r="A10" t="s">
-        <v>36</v>
-      </c>
-      <c r="B10" t="s">
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C10" t="s">
+      <c r="B11" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D10" t="s">
-        <v>38</v>
-      </c>
-      <c r="E10" t="s">
-        <v>14</v>
-      </c>
-      <c r="F10" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="A11" t="s">
+      <c r="D11" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B11" t="s">
+      <c r="E11" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C11" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="F11" s="5" t="s">
         <v>41</v>
-      </c>
-      <c r="E11" t="s">
-        <v>42</v>
-      </c>
-      <c r="F11" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>
   <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
@@ -1108,7 +1184,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5DE3A5DC-D32E-4FDD-A31F-2EDF54B09E4E}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{3331F6D5-ECFB-4E51-94CB-62BCD35402DC}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -1123,425 +1199,425 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" t="s">
         <v>49</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>50</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" t="s">
         <v>51</v>
       </c>
-      <c r="D2" t="s">
-        <v>52</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H2" t="s">
         <v>53</v>
-      </c>
-      <c r="F2" t="s">
-        <v>54</v>
-      </c>
-      <c r="G2" t="s">
-        <v>54</v>
-      </c>
-      <c r="H2" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" t="s">
         <v>56</v>
       </c>
-      <c r="B3" t="s">
+      <c r="E3" t="s">
         <v>57</v>
       </c>
-      <c r="C3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D3" t="s">
-        <v>58</v>
-      </c>
-      <c r="E3" t="s">
-        <v>59</v>
-      </c>
       <c r="F3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" t="s">
         <v>60</v>
       </c>
-      <c r="B4" t="s">
+      <c r="E4" t="s">
         <v>61</v>
       </c>
-      <c r="C4" t="s">
-        <v>51</v>
-      </c>
-      <c r="D4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E4" t="s">
-        <v>63</v>
-      </c>
       <c r="F4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" t="s">
         <v>64</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" t="s">
         <v>65</v>
       </c>
-      <c r="C5" t="s">
+      <c r="E5" t="s">
         <v>66</v>
       </c>
-      <c r="D5" t="s">
-        <v>67</v>
-      </c>
-      <c r="E5" t="s">
-        <v>68</v>
-      </c>
       <c r="F5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D6" t="s">
         <v>69</v>
       </c>
-      <c r="B6" t="s">
+      <c r="E6" t="s">
         <v>70</v>
       </c>
-      <c r="C6" t="s">
-        <v>66</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="F6" t="s">
         <v>71</v>
       </c>
-      <c r="E6" t="s">
-        <v>72</v>
-      </c>
-      <c r="F6" t="s">
-        <v>73</v>
-      </c>
       <c r="G6" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H6" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" t="s">
+        <v>72</v>
+      </c>
+      <c r="B7" t="s">
+        <v>73</v>
+      </c>
+      <c r="C7" t="s">
         <v>74</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
         <v>75</v>
       </c>
-      <c r="C7" t="s">
+      <c r="E7" t="s">
         <v>76</v>
       </c>
-      <c r="D7" t="s">
-        <v>77</v>
-      </c>
-      <c r="E7" t="s">
-        <v>78</v>
-      </c>
       <c r="F7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C8" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" t="s">
         <v>79</v>
       </c>
-      <c r="B8" t="s">
-        <v>80</v>
-      </c>
-      <c r="C8" t="s">
-        <v>76</v>
-      </c>
-      <c r="D8" t="s">
-        <v>81</v>
-      </c>
       <c r="E8" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C9" t="s">
+        <v>74</v>
+      </c>
+      <c r="D9" t="s">
         <v>82</v>
       </c>
-      <c r="B9" t="s">
+      <c r="E9" t="s">
         <v>83</v>
       </c>
-      <c r="C9" t="s">
-        <v>76</v>
-      </c>
-      <c r="D9" t="s">
-        <v>84</v>
-      </c>
-      <c r="E9" t="s">
-        <v>85</v>
-      </c>
       <c r="F9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" t="s">
+        <v>84</v>
+      </c>
+      <c r="B10" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" t="s">
         <v>86</v>
       </c>
-      <c r="B10" t="s">
+      <c r="E10" t="s">
         <v>87</v>
       </c>
-      <c r="C10" t="s">
-        <v>76</v>
-      </c>
-      <c r="D10" t="s">
-        <v>88</v>
-      </c>
-      <c r="E10" t="s">
-        <v>89</v>
-      </c>
       <c r="F10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" t="s">
+        <v>88</v>
+      </c>
+      <c r="B11" t="s">
+        <v>89</v>
+      </c>
+      <c r="C11" t="s">
+        <v>74</v>
+      </c>
+      <c r="D11" t="s">
         <v>90</v>
       </c>
-      <c r="B11" t="s">
+      <c r="E11" t="s">
         <v>91</v>
       </c>
-      <c r="C11" t="s">
-        <v>76</v>
-      </c>
-      <c r="D11" t="s">
-        <v>92</v>
-      </c>
-      <c r="E11" t="s">
-        <v>93</v>
-      </c>
       <c r="F11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" t="s">
+        <v>93</v>
+      </c>
+      <c r="C12" t="s">
         <v>94</v>
       </c>
-      <c r="B12" t="s">
+      <c r="D12" t="s">
         <v>95</v>
       </c>
-      <c r="C12" t="s">
+      <c r="E12" t="s">
         <v>96</v>
       </c>
-      <c r="D12" t="s">
-        <v>97</v>
-      </c>
-      <c r="E12" t="s">
-        <v>98</v>
-      </c>
       <c r="F12" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G12" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H12" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" t="s">
+        <v>97</v>
+      </c>
+      <c r="B13" t="s">
+        <v>98</v>
+      </c>
+      <c r="C13" t="s">
+        <v>94</v>
+      </c>
+      <c r="D13" t="s">
         <v>99</v>
       </c>
-      <c r="B13" t="s">
-        <v>100</v>
-      </c>
-      <c r="C13" t="s">
-        <v>96</v>
-      </c>
-      <c r="D13" t="s">
-        <v>101</v>
-      </c>
       <c r="E13" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" t="s">
+        <v>100</v>
+      </c>
+      <c r="B14" t="s">
+        <v>101</v>
+      </c>
+      <c r="C14" t="s">
+        <v>94</v>
+      </c>
+      <c r="D14" t="s">
         <v>102</v>
       </c>
-      <c r="B14" t="s">
+      <c r="E14" t="s">
         <v>103</v>
       </c>
-      <c r="C14" t="s">
-        <v>96</v>
-      </c>
-      <c r="D14" t="s">
-        <v>104</v>
-      </c>
-      <c r="E14" t="s">
-        <v>105</v>
-      </c>
       <c r="F14" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G14" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H14" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" t="s">
+        <v>104</v>
+      </c>
+      <c r="B15" t="s">
+        <v>105</v>
+      </c>
+      <c r="C15" t="s">
         <v>106</v>
       </c>
-      <c r="B15" t="s">
+      <c r="D15" t="s">
         <v>107</v>
       </c>
-      <c r="C15" t="s">
+      <c r="E15" t="s">
         <v>108</v>
       </c>
-      <c r="D15" t="s">
-        <v>109</v>
-      </c>
-      <c r="E15" t="s">
-        <v>110</v>
-      </c>
       <c r="F15" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G15" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H15" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" t="s">
+        <v>109</v>
+      </c>
+      <c r="B16" t="s">
+        <v>110</v>
+      </c>
+      <c r="C16" t="s">
+        <v>94</v>
+      </c>
+      <c r="D16" t="s">
         <v>111</v>
       </c>
-      <c r="B16" t="s">
+      <c r="E16" t="s">
         <v>112</v>
       </c>
-      <c r="C16" t="s">
-        <v>96</v>
-      </c>
-      <c r="D16" t="s">
-        <v>113</v>
-      </c>
-      <c r="E16" t="s">
-        <v>114</v>
-      </c>
       <c r="F16" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G16" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="H16" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
   <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
@@ -1554,7 +1630,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{5A14ACD7-EA54-495F-A726-BDDC6FFE75F2}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{DB1B6729-FF59-4E51-8D2C-CF39801FB60D}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
@@ -1567,100 +1643,100 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="E1" s="2" t="s">
+      <c r="D1" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C2" t="s">
         <v>116</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E2" t="s">
         <v>117</v>
       </c>
-      <c r="C2" t="s">
+      <c r="F2" t="s">
         <v>118</v>
-      </c>
-      <c r="D2" t="s">
-        <v>94</v>
-      </c>
-      <c r="E2" t="s">
-        <v>119</v>
-      </c>
-      <c r="F2" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C3" t="s">
+        <v>116</v>
+      </c>
+      <c r="D3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E3" t="s">
+        <v>117</v>
+      </c>
+      <c r="F3" t="s">
         <v>118</v>
-      </c>
-      <c r="D3" t="s">
-        <v>99</v>
-      </c>
-      <c r="E3" t="s">
-        <v>119</v>
-      </c>
-      <c r="F3" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B4" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E4" t="s">
+        <v>117</v>
+      </c>
+      <c r="F4" t="s">
         <v>118</v>
-      </c>
-      <c r="D4" t="s">
-        <v>102</v>
-      </c>
-      <c r="E4" t="s">
-        <v>119</v>
-      </c>
-      <c r="F4" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" t="s">
+        <v>123</v>
+      </c>
+      <c r="B5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C5" t="s">
         <v>125</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" t="s">
+        <v>92</v>
+      </c>
+      <c r="E5" t="s">
         <v>126</v>
-      </c>
-      <c r="C5" t="s">
-        <v>127</v>
-      </c>
-      <c r="D5" t="s">
-        <v>94</v>
-      </c>
-      <c r="E5" t="s">
-        <v>128</v>
       </c>
       <c r="F5" t="s">
         <v>10</v>
@@ -1668,19 +1744,19 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B6" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C6" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E6" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F6" t="s">
         <v>10</v>
@@ -1688,19 +1764,19 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B7" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C7" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D7" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E7" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F7" t="s">
         <v>10</v>
@@ -1708,19 +1784,19 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B8" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E8" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F8" t="s">
         <v>10</v>
@@ -1728,19 +1804,19 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B9" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D9" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E9" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F9" t="s">
         <v>10</v>
@@ -1748,19 +1824,19 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B10" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C10" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D10" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E10" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F10" t="s">
         <v>10</v>
@@ -1768,19 +1844,19 @@
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B11" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C11" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D11" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E11" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F11" t="s">
         <v>10</v>
@@ -1789,7 +1865,7 @@
   </sheetData>
   <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
@@ -1799,4 +1875,199 @@
   </tableParts>
   <extLst/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{F3442743-9BE2-4748-B226-D7296D337312}" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:T200"/>
+  <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="12"/>
+      <c r="E1" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="11">
+        <v>12345</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1">
+      <c r="A5" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="15">
+        <v>999999999999999</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="16" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
+  </headerFooter>
+  <extLst/>
+</worksheet>
 </file>
</xml_diff>